<commit_message>
feat: Add Excel and CSV parsing utilities with data merging logic and VS Code debug configurations.
</commit_message>
<xml_diff>
--- a/testcase/MergeTest.xlsx
+++ b/testcase/MergeTest.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="20">
   <si>
     <t>#MergeTest</t>
   </si>
@@ -44,12 +44,18 @@
     <t>测试不被合并进去</t>
   </si>
   <si>
+    <t>测试物品二级合并</t>
+  </si>
+  <si>
     <t>merged_arr</t>
   </si>
   <si>
     <t>normal_col</t>
   </si>
   <si>
+    <t>merged_arr2</t>
+  </si>
+  <si>
     <t>$</t>
   </si>
   <si>
@@ -63,6 +69,15 @@
   </si>
   <si>
     <t>string</t>
+  </si>
+  <si>
+    <t>Item[]</t>
+  </si>
+  <si>
+    <t>Id</t>
+  </si>
+  <si>
+    <t>Count</t>
   </si>
   <si>
     <t>test1</t>
@@ -692,10 +707,17 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1080,15 +1102,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:E8"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelRow="7" outlineLevelCol="4"/>
+  <dimension ref="A1:I14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:9">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:9">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -1102,93 +1124,189 @@
       <c r="E2" t="s">
         <v>4</v>
       </c>
+      <c r="F2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:9">
       <c r="B3" t="s">
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E3" t="s">
-        <v>6</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:9">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C4" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E4" t="s">
-        <v>8</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:9">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+      <c r="I5" s="2"/>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" t="s">
+        <v>1</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="B7">
+        <v>1001</v>
+      </c>
+      <c r="C7">
         <v>10</v>
       </c>
-      <c r="E5" t="s">
-        <v>11</v>
+      <c r="D7">
+        <v>20</v>
+      </c>
+      <c r="E7" t="s">
+        <v>17</v>
+      </c>
+      <c r="F7" s="3">
+        <v>10001</v>
+      </c>
+      <c r="G7">
+        <v>1</v>
+      </c>
+      <c r="H7" s="3">
+        <v>10004</v>
+      </c>
+      <c r="I7">
+        <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
-      <c r="B6">
-        <v>1001</v>
-      </c>
-      <c r="C6">
-        <v>10</v>
-      </c>
-      <c r="D6">
-        <v>20</v>
-      </c>
-      <c r="E6" t="s">
-        <v>12</v>
+    <row r="8" spans="1:9">
+      <c r="B8">
+        <v>1002</v>
+      </c>
+      <c r="C8">
+        <v>30</v>
+      </c>
+      <c r="E8" t="s">
+        <v>18</v>
+      </c>
+      <c r="F8" s="3">
+        <v>10002</v>
+      </c>
+      <c r="G8">
+        <v>2</v>
+      </c>
+      <c r="H8" s="3">
+        <v>10005</v>
+      </c>
+      <c r="I8">
+        <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
-      <c r="B7">
-        <v>1002</v>
-      </c>
-      <c r="C7">
-        <v>30</v>
-      </c>
-      <c r="E7" t="s">
-        <v>13</v>
+    <row r="9" spans="1:9">
+      <c r="B9">
+        <v>1003</v>
+      </c>
+      <c r="D9">
+        <v>40</v>
+      </c>
+      <c r="E9" t="s">
+        <v>19</v>
+      </c>
+      <c r="F9" s="3">
+        <v>10003</v>
+      </c>
+      <c r="G9">
+        <v>3</v>
+      </c>
+      <c r="H9" s="3">
+        <v>10006</v>
+      </c>
+      <c r="I9">
+        <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
-      <c r="B8">
-        <v>1003</v>
-      </c>
-      <c r="D8">
-        <v>40</v>
-      </c>
-      <c r="E8" t="s">
-        <v>14</v>
-      </c>
+    <row r="10" spans="1:9">
+      <c r="F10" s="4"/>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="F11" s="4"/>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="F12" s="4"/>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="F13" s="4"/>
+    </row>
+    <row r="14" spans="1:9">
+      <c r="F14" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="8">
     <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:I2"/>
     <mergeCell ref="C3:D3"/>
+    <mergeCell ref="F3:I3"/>
     <mergeCell ref="C4:D4"/>
+    <mergeCell ref="F4:I4"/>
     <mergeCell ref="C5:D5"/>
+    <mergeCell ref="F5:I5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
   <ignoredErrors>
-    <ignoredError sqref="C1:E1 B3:E8" numberStoredAsText="1"/>
+    <ignoredError sqref="B7:E9 B3:E5 C1:E1" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>